<commit_message>
Consolidate recruiter catalog to 162 unique sites
Merge sources:
- Original 20 hand-classified recruiters
- 118 names from OneClickHustle's Company filter (4 agent research batches)
- ~95 unique entries from the user's recruiter dump (2 more agent batches)

Dedup by canonical domain (162 unique sites after collapsing aliases like
Field Goals -> The Heard, Think Group -> Become A Thinker, Schlesinger ->
SAGO, Murray Hill Center -> Murray Hill National).

Classification breakdown:
- 34 Browsable (public)
- 21 Browsable (login)
- 1 Browsable (mobile app)
- 24 Unclear (login required to verify)
- 82 Email-only (no scraper needed; covered by inbox scanning)

The 56 Browsable-class recruiters are the candidates for scraper
extractors; the 82 Email-only are out of scraping scope. The 24 Unclear
need a manual logged-in check to confirm.
</commit_message>
<xml_diff>
--- a/docs/recruiters.xlsx
+++ b/docs/recruiters.xlsx
@@ -422,12 +422,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="62" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -450,228 +450,228 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Accelerant Research</t>
+          <t>10K Voices</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Browsable</t>
+          <t>Unclear</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>https://www.accelerantresearch.com/availableresearch</t>
+          <t>https://community.10kvoices.com</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Reckner</t>
+          <t>20/20 Panel</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Email-only</t>
+          <t>Unclear</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>https://www.reckner.com</t>
+          <t>https://join.2020panel.com/</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>The Heard</t>
+          <t>Accelerant Research</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Email-only</t>
+          <t>Browsable</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>https://www.betheheard.com</t>
+          <t>https://www.accelerantresearch.com/availableresearch</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Opinions Link</t>
+          <t>Act One Research</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Email-only</t>
+          <t>Unclear</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>https://www.opinionslink.com</t>
+          <t>https://www.actone-research.com</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Opinions by Sync</t>
+          <t>Adler Weiner Research</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Browsable</t>
+          <t>Email-only</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>https://community.opinionsbysync.com/s/Jobsite</t>
+          <t>https://adlerweiner.com</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Galloway Research</t>
+          <t>Advanced Focus</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Browsable</t>
+          <t>Unclear</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>https://www.questionspace.net/category/upcoming-studies/</t>
+          <t>https://ow.advancedfocus.com</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>User Interviews</t>
+          <t>Advanced Opinions</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Browsable</t>
+          <t>Unclear</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>https://www.userinterviews.com/studies</t>
+          <t>http://register.advancedopinions.com</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Daisy Mae Research</t>
+          <t>Amplify Research</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Browsable</t>
+          <t>Email-only</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>https://daisymaeresearch.com/projects/</t>
+          <t>https://amplifyresearch.com/participate/</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>PRC</t>
+          <t>Ann Michaels / iShopForYou</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Browsable</t>
+          <t>Browsable (login)</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>https://www.prcmarketresearch.com/upcomingprojects</t>
+          <t>https://ishopforyou.com/evaluator-login</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Nelson Recruiting</t>
+          <t>Apex Focus Group</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Email-only</t>
+          <t>Browsable</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>https://nelsonrecruiting.com</t>
+          <t>https://apexfocusgroup.com/</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>User Research International</t>
+          <t>Ascendancy Research</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Browsable (login)</t>
+          <t>Browsable</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>https://app.uriux.com/studies</t>
+          <t>https://studies.ascendresearch.com/</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Become A Thinker</t>
+          <t>Askable</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Browsable</t>
+          <t>Unclear</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>https://becomeathinker.com/upcoming-studies/</t>
+          <t>https://www.askable.com/earn/participants</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>10K Voices</t>
+          <t>ATH Power Consulting</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Unclear</t>
+          <t>Browsable (login)</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>https://community.10kvoices.com</t>
+          <t>https://experienceapc.com/getting-started</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Adler Weiner Research</t>
+          <t>Atkins Research</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -681,109 +681,2511 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>https://adlerweiner.com</t>
+          <t>https://www.atkinsresearch.com/research-participant/respondent-signup/</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Advanced Focus</t>
+          <t>Become A Thinker</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Unclear</t>
+          <t>Browsable</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>https://ow.advancedfocus.com</t>
+          <t>https://becomeathinker.com/upcoming-studies/</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Advanced Opinions</t>
+          <t>BestMark</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Unclear</t>
+          <t>Browsable (login)</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>http://register.advancedopinions.com</t>
+          <t>https://secure.bestmark.com/public/application/appstart.aspx</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Respondent</t>
+          <t>Bezel Research</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Browsable (login)</t>
+          <t>Email-only</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>https://app.respondent.io/respondents/v2/projects/browse</t>
+          <t>http://bezelrr.com/</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Prolific</t>
+          <t>Big Bang Recruiting</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Browsable (login)</t>
+          <t>Email-only</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>https://app.prolific.com/</t>
+          <t>https://www.bigbangrecruiting.com/register/</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>dscout</t>
+          <t>Blink UX</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Browsable (mobile app)</t>
+          <t>Unclear</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>https://dscout.com</t>
+          <t>https://participate.blinkux.com/</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
+          <t>Brightside Research Solutions</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>https://teambrightsider.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Cambridge Focus</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>http://www.participatenewengland.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Cara Casting</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Browsable</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>https://jobs.caracasting.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>CIC Testing</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cictesting.com/CIC/</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Citrus Labs</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>https://www.citruslabs.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>ClearView Research</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>http://www.clearviewresearch.com/sign-up-now.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Collab Research</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>https://www.collab-research.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Compass Research</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>https://compassmarketingresearch.com/sign-up/</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Confide Research</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>https://confideresearch.com/Participants/signup</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>ConneXion Research</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Browsable</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>https://jointheconnexion.com/current-projects/</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Consumer Viewpoint</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>https://www.paidforyouropinions.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Contact Design</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>https://yourcontacthub.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Contract Testing</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>https://connect.contracttesting.com/ctimvc/Account/Register</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Unclear</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Curion</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Browsable (login)</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>https://curionpanelist.com/portal/default</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Cypher Research</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>https://cypherresearch.com/intranet/respondent_sign_up.php</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Daisy Mae Research</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Browsable</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>https://daisymaeresearch.com/projects/</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Decision Point Research</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>https://www.decisionpointresearch.ca</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Design Science</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>https://dscience.com/signup</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Drive Research</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>https://www.driveresearch.com/participate/</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>dscout</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Browsable (mobile app)</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>https://dscout.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Elliott Benson</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>https://www.elliottbenson.com/participate/</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>End to End Research</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Unclear</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>https://www.endtoenduserresearch.com/participate.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Engage In Depth</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>https://engageindepth.com/participate/</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Ethical Mind</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>https://ethicalmind.org/</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>FF Focus Group</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Browsable</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>https://www.fffocusgroup.com/current-projects/</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Field Agent / Storesight</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Browsable (login)</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>https://app.fieldagent.net/</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Field Voices</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Browsable</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>https://fieldvoices.com/current_studies</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
           <t>Fieldwork</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Email-only</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
         <is>
           <t>https://www.fieldwork.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>First Court Jurors</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>https://www.firstcourt.com/jury-recruiting</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Fleischman Field Research</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>http://www.ffrsf.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Focus &amp; Testing</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>https://research.focusandtesting.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>focus 99</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>https://www.focus99.com/sub/</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Focus Corner</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>https://focuscorner.net/</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Focus Crossroads</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>https://focuscrossroads.org/research-network/join-consumer/</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Focus Group Connection</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>https://www.focusgroupconnection.com/participate/</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Focus Group Panel</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Browsable</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>https://focusgrouppanel.com/research-category/focus-group/</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Focus Insite</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Unclear</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>https://linktr.ee/focus_insite</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Focus Pulse</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>https://focuspulseresearch.co.uk/</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Focus Room</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Browsable</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>https://focusroom.com/active-studies/</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Focuscope</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>https://www.focuscope.com/join-our-community/</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Funds for Focus</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Unclear</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>https://fundsforfocus.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Galloway Research</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Browsable</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>https://www.questionspace.net/category/upcoming-studies/</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Georgetown University (GRVP)</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>https://grvp.georgetown.edu/</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Good Gamer Group</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Browsable</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>https://goodgamergroup.com/available-studies/</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Griot Recruit</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>https://www.griotrecruit.co/</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Hagen Sinclair Research Recruiting</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>https://hagensinclair.com/paid-research-studies-2/</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Horizon Group</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>https://www.horizongroupiowa.com/join-our-panel/</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>IDEO Design Research</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Browsable</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>https://designresearch.ideo.com/opportunities</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Insight Recruit</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>https://insightrecruit.com/join-our-panel/</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Intact Qualitative Research</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>https://www.iqrsf.com/participant-intake-form</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>ISG (Information Specialists Group)</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Unclear</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>http://www.isgpanel.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Ivy Exec</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Browsable (login)</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>https://ivyexec.com/jobs-and-research-studies-search?type=study</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Jackson Associates</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Browsable (login)</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>https://research.jacksonassociates.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>JC Research Partners</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>https://jcresearchpartners.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>JJA Research</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Browsable</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>https://jjarecruiting.com/?post_type=project</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>KSS International</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Browsable (login)</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>http://kernscheduling.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>L&amp;E Research</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Browsable (login)</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>https://www.leopinions.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Leede Research</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Browsable</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t>https://leedemn.com/join-our-database/available-studies/</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Lees Focus</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Browsable</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>https://leesfocusgroups.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Limelight by Shugoll</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>https://limelightbyshugoll.com/get-paid-for-your-opinion/</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Local Focus Group</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>https://www.localfocusgroup.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>MacConnell Research</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Unclear</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="inlineStr">
+        <is>
+          <t>http://www.macconnellresearch.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Market-Ease (Market Eaze)</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Browsable</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>https://www.market-ease.com/about-the-respondent-hub</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>MarketForce</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Browsable (login)</t>
+        </is>
+      </c>
+      <c r="C85" s="2" t="inlineStr">
+        <is>
+          <t>https://shopper.marketforce.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Mars Research</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>https://joinmarsresearch.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>McCormick Group</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C87" s="2" t="inlineStr">
+        <is>
+          <t>http://mccormick-group.com/market-research.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Mediabarn Research</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Browsable</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mediabarnresearch.com/currentstudies/</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>MeThinks</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Browsable (login)</t>
+        </is>
+      </c>
+      <c r="C89" s="2" t="inlineStr">
+        <is>
+          <t>https://www.methinks.io/thinker</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>MForce Research</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>http://www.mforceresearch.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Mindswarms</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Browsable (login)</t>
+        </is>
+      </c>
+      <c r="C91" s="2" t="inlineStr">
+        <is>
+          <t>https://app.mindswarms.com/sign_in</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Moore Opinions</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t>http://mooreopinions.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Moore Research Services</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C93" s="2" t="inlineStr">
+        <is>
+          <t>https://www.moore-research.com/join-a-panel/</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Murray Hill National</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Unclear</t>
+        </is>
+      </c>
+      <c r="C94" s="2" t="inlineStr">
+        <is>
+          <t>https://panels.murrayhillnational.com/Portal/Default</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>MVG Recruiting</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C95" s="2" t="inlineStr">
+        <is>
+          <t>https://mvgrecruiting.com/sign-up</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>N.C. Litigation &amp; Jury Research Group</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C96" s="2" t="inlineStr">
+        <is>
+          <t>https://ncfocusgroups.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Nashville Research Group</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Browsable</t>
+        </is>
+      </c>
+      <c r="C97" s="2" t="inlineStr">
+        <is>
+          <t>https://www.nashvilleresearch.com/current-research-projects</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Nationwide Research Recruiters</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Browsable</t>
+        </is>
+      </c>
+      <c r="C98" s="2" t="inlineStr">
+        <is>
+          <t>https://www.nwrrs.com/focus-group-calendar.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>NDR (National Data Research)</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Unclear</t>
+        </is>
+      </c>
+      <c r="C99" s="2" t="inlineStr">
+        <is>
+          <t>http://www.national-data.net/</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Nelson Recruiting</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C100" s="2" t="inlineStr">
+        <is>
+          <t>https://nelsonrecruiting.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>New England Focus Group</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C101" s="2" t="inlineStr">
+        <is>
+          <t>https://www.newenglandfocusgroup.com/register.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Newton (ambiguous)</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Unclear</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr"/>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Newton Marketing Network</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C103" s="2" t="inlineStr">
+        <is>
+          <t>https://newtonmarketingnetwork.com/participants/</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Nichols Research</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C104" s="2" t="inlineStr">
+        <is>
+          <t>https://nicholsresearch.com/registration-form/</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>NYC Focal (The Diamond Lists)</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C105" s="2" t="inlineStr">
+        <is>
+          <t>https://thediamondlists.com/join-the-list/</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Olympic National Research</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Unclear</t>
+        </is>
+      </c>
+      <c r="C106" s="2" t="inlineStr">
+        <is>
+          <t>https://olympicnationalprojects.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Online Verdict</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C107" s="2" t="inlineStr">
+        <is>
+          <t>https://www.onlineverdict.com/jurors/signup/</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Opinions by Sync</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Browsable</t>
+        </is>
+      </c>
+      <c r="C108" s="2" t="inlineStr">
+        <is>
+          <t>https://community.opinionsbysync.com/s/Jobsite</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Opinions for Cash</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Unclear</t>
+        </is>
+      </c>
+      <c r="C109" s="2" t="inlineStr">
+        <is>
+          <t>https://opinionsforcash.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Opinions Link</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C110" s="2" t="inlineStr">
+        <is>
+          <t>https://www.opinionslink.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Opinions LTD</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C111" s="2" t="inlineStr">
+        <is>
+          <t>https://www.opinionsltd.com/participate/</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Orman Guidance</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Browsable</t>
+        </is>
+      </c>
+      <c r="C112" s="2" t="inlineStr">
+        <is>
+          <t>https://ormanguidance.com/participate/projects/</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>People for Research</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Browsable (login)</t>
+        </is>
+      </c>
+      <c r="C113" s="2" t="inlineStr">
+        <is>
+          <t>https://www.peopleforresearch.co.uk/participant/opportunities</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>Portable Insights</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C114" s="2" t="inlineStr">
+        <is>
+          <t>https://portableinsights.com/join-our-panel</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Pragmatic Research</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Unclear</t>
+        </is>
+      </c>
+      <c r="C115" s="2" t="inlineStr">
+        <is>
+          <t>http://www.pragmatic-research.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>PRC</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Browsable</t>
+        </is>
+      </c>
+      <c r="C116" s="2" t="inlineStr">
+        <is>
+          <t>https://www.prcmarketresearch.com/upcomingprojects</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>Precision Research</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C117" s="2" t="inlineStr">
+        <is>
+          <t>https://www.opinionwizard.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>Prepare to Persuade</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Unclear</t>
+        </is>
+      </c>
+      <c r="C118" s="2" t="inlineStr">
+        <is>
+          <t>https://www.preparetopersuade.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>Private Jury</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Browsable</t>
+        </is>
+      </c>
+      <c r="C119" s="2" t="inlineStr">
+        <is>
+          <t>https://www.privatejury.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>Probe Market Research</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>Browsable</t>
+        </is>
+      </c>
+      <c r="C120" s="2" t="inlineStr">
+        <is>
+          <t>https://www.probemarket.com/available-studies/</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>Product Tube</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C121" s="2" t="inlineStr">
+        <is>
+          <t>https://web.producttube.com/signup</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>Prolific</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>Browsable (login)</t>
+        </is>
+      </c>
+      <c r="C122" s="2" t="inlineStr">
+        <is>
+          <t>https://app.prolific.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>PVR Research</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C123" s="2" t="inlineStr">
+        <is>
+          <t>http://www.pvr-research.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>Q-Insights</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C124" s="2" t="inlineStr">
+        <is>
+          <t>https://q-insights.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>Qual Recruit</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C125" s="2" t="inlineStr">
+        <is>
+          <t>https://www.qualrecruit.com/become-a-participant</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>Rare Patient Voice</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Browsable</t>
+        </is>
+      </c>
+      <c r="C126" s="2" t="inlineStr">
+        <is>
+          <t>https://rarepatientvoice.com/for-patients/study-opportunities/</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>Real Focus Group</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Browsable</t>
+        </is>
+      </c>
+      <c r="C127" s="2" t="inlineStr">
+        <is>
+          <t>https://realfocusgroup.com/upcoming/</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>Reckner</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C128" s="2" t="inlineStr">
+        <is>
+          <t>https://www.reckner.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>Recruit and Field</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C129" s="2" t="inlineStr">
+        <is>
+          <t>https://www.recruitandfield.com/register-as-a-participant</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>Research America</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>Unclear</t>
+        </is>
+      </c>
+      <c r="C130" s="2" t="inlineStr">
+        <is>
+          <t>https://researchamericainc.net/</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>Research Outloud</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C131" s="2" t="inlineStr">
+        <is>
+          <t>https://researchoutloud.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>Respondent</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Browsable (login)</t>
+        </is>
+      </c>
+      <c r="C132" s="2" t="inlineStr">
+        <is>
+          <t>https://app.respondent.io/respondents/v2/projects/browse</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>Ridgeline Recruiting</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C133" s="2" t="inlineStr">
+        <is>
+          <t>https://ridgelinerecruiting.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>Round2Research</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C134" s="2" t="inlineStr">
+        <is>
+          <t>https://round2research.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>RRU Research</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C135" s="2" t="inlineStr">
+        <is>
+          <t>https://focuspocussoftware.net/WP_RRU/Register</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>SAGO (Schlesinger / Focus Pointe Global)</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>Browsable (login)</t>
+        </is>
+      </c>
+      <c r="C136" s="2" t="inlineStr">
+        <is>
+          <t>https://www.focusgroup.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>Savvy Cooperative</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>Browsable (login)</t>
+        </is>
+      </c>
+      <c r="C137" s="2" t="inlineStr">
+        <is>
+          <t>https://apply.savvy.coop/</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>Secret Shopper</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Browsable (login)</t>
+        </is>
+      </c>
+      <c r="C138" s="2" t="inlineStr">
+        <is>
+          <t>https://www.secretshopper.com/shoppers/shoppers</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>SIS Research</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C139" s="2" t="inlineStr">
+        <is>
+          <t>https://participate.sisinternational.com/Portal/Default</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>Spotlight Research</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C140" s="2" t="inlineStr">
+        <is>
+          <t>https://spotlightmarketresearch.com/join-our-audience/</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>Take Part in Research</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>Browsable</t>
+        </is>
+      </c>
+      <c r="C141" s="2" t="inlineStr">
+        <is>
+          <t>https://takepartinresearch.co.uk/current-projects/</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>Talking Heads</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C142" s="2" t="inlineStr">
+        <is>
+          <t>http://register.talkingheadsstudio.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>Taylor Research</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>Unclear</t>
+        </is>
+      </c>
+      <c r="C143" s="2" t="inlineStr">
+        <is>
+          <t>https://studies.taylorresearch.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>The Heard</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>Browsable</t>
+        </is>
+      </c>
+      <c r="C144" s="2" t="inlineStr">
+        <is>
+          <t>https://www.betheheard.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>The Insighters</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>Browsable</t>
+        </is>
+      </c>
+      <c r="C145" s="2" t="inlineStr">
+        <is>
+          <t>https://theinsighters.com/public-opportunities</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>The Social Question</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>Browsable</t>
+        </is>
+      </c>
+      <c r="C146" s="2" t="inlineStr">
+        <is>
+          <t>https://www.the-socialq.com/open-studies</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>Theoretics</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>Browsable</t>
+        </is>
+      </c>
+      <c r="C147" s="2" t="inlineStr">
+        <is>
+          <t>https://www.theoretics.co/current-projects</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>TrendSource</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>Browsable (login)</t>
+        </is>
+      </c>
+      <c r="C148" s="2" t="inlineStr">
+        <is>
+          <t>https://www.thesourceagents.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>Truscott Research</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>Unclear</t>
+        </is>
+      </c>
+      <c r="C149" s="2" t="inlineStr">
+        <is>
+          <t>https://app.truscottresearch.com/register</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>Ubinsights</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C150" s="2" t="inlineStr">
+        <is>
+          <t>https://ubinsights.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>Uncover Research</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C151" s="2" t="inlineStr">
+        <is>
+          <t>https://www.uncoverresearch.com/participate</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>User Insight</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C152" s="2" t="inlineStr">
+        <is>
+          <t>https://www.shareyourinsights.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>User Interviews</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>Browsable</t>
+        </is>
+      </c>
+      <c r="C153" s="2" t="inlineStr">
+        <is>
+          <t>https://www.userinterviews.com/studies</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>User Research International</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>Browsable (login)</t>
+        </is>
+      </c>
+      <c r="C154" s="2" t="inlineStr">
+        <is>
+          <t>https://app.uriux.com/studies</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>uTest</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Browsable (login)</t>
+        </is>
+      </c>
+      <c r="C155" s="2" t="inlineStr">
+        <is>
+          <t>https://www.utest.com/projects</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>Videochat Network</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C156" s="2" t="inlineStr">
+        <is>
+          <t>https://www.videochatnetwork.net/sign-up/</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>View-Finders</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C157" s="2" t="inlineStr">
+        <is>
+          <t>https://www.view-finders.net/participant-registration-2/</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>WAC Research</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C158" s="2" t="inlineStr">
+        <is>
+          <t>https://wacresearch.com/data.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>Watch Me Think</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C159" s="2" t="inlineStr">
+        <is>
+          <t>https://watchmethink.com/contribute</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>Watchlab</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C160" s="2" t="inlineStr">
+        <is>
+          <t>https://watchlab.com/sign-up/</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>When Opinions Meet</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>Unclear</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr"/>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>Wilkins Research Services</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C162" s="2" t="inlineStr">
+        <is>
+          <t>https://wilkinsresearch.net/join-our-panel/</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>Winn Winn Research</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C163" s="2" t="inlineStr">
+        <is>
+          <t>https://winnwinn.com/new/public/register</t>
         </is>
       </c>
     </row>
@@ -809,6 +3211,145 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId18"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId19"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C33" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C35" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C36" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C37" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C38" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C39" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C40" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C41" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C42" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C43" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C44" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C45" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C46" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C47" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C48" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C49" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C50" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C51" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C52" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C53" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C54" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C55" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C56" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C57" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C58" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C59" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C60" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C61" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C62" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C63" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C64" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C65" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C66" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C67" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C68" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C69" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C70" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C71" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C72" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C73" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C74" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C75" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C76" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C77" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C78" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C79" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C80" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C81" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C82" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C83" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C84" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C85" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C86" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C87" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C88" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C89" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C90" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C91" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C92" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C93" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C94" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C95" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C96" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C97" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C98" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C99" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C100" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C101" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C103" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C104" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C105" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C106" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C107" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C108" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C109" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C110" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C111" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C112" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C113" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C114" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C115" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C116" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C117" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C118" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C119" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C120" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C121" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C122" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C123" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C124" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C125" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C126" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C127" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C128" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C129" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C130" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C131" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C132" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C133" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C134" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C135" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C136" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C137" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C138" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C139" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C140" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C141" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C142" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C143" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C144" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C145" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C146" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C147" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C148" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C149" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C150" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C151" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C152" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C153" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C154" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C155" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C156" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C157" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C158" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C159" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C160" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C162" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C163" r:id="rId159"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add 10 recruiters discovered via Gmail scan
Gmail search of the past 12 months surfaced 10 active recruiters not
present in the OneClickHustle-sourced catalog. Highest volume by far
was Pulse Labs (22 threads — multiple study programs running through
2025-2026). Others are smaller-volume but legitimate: Focus Group
Finder, AlphaBuzz, EmCee Research, Thurs Recruiting, Wynter, AMG
Research, TELUS Digital, VGM, CEC Surveys.

Three Gmail finds were skipped as duplicates / not recruiters:
- Think Group Austin (already covered by Become A Thinker)
- Insight Space (rebranded as Blink Recruiting, already in catalog)
- Discuss.io (video-chat platform, not a recruiter)

Catalog now: 172 unique recruiters (34 browsable, 22 browsable-login,
1 mobile app, 26 unclear, 89 email-only).
</commit_message>
<xml_diff>
--- a/docs/recruiters.xlsx
+++ b/docs/recruiters.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C163"/>
+  <dimension ref="A1:C173"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -569,7 +569,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Amplify Research</t>
+          <t>AlphaBuzz</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -579,201 +579,201 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>https://amplifyresearch.com/participate/</t>
+          <t>https://alphabuzz.alchemer.com/</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Ann Michaels / iShopForYou</t>
+          <t>AMG Research</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Browsable (login)</t>
+          <t>Email-only</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>https://ishopforyou.com/evaluator-login</t>
+          <t>https://amgsurvey.com/</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Apex Focus Group</t>
+          <t>Amplify Research</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Browsable</t>
+          <t>Email-only</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>https://apexfocusgroup.com/</t>
+          <t>https://amplifyresearch.com/participate/</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Ascendancy Research</t>
+          <t>Ann Michaels / iShopForYou</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Browsable</t>
+          <t>Browsable (login)</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>https://studies.ascendresearch.com/</t>
+          <t>https://ishopforyou.com/evaluator-login</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Askable</t>
+          <t>Apex Focus Group</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Unclear</t>
+          <t>Browsable</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>https://www.askable.com/earn/participants</t>
+          <t>https://apexfocusgroup.com/</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ATH Power Consulting</t>
+          <t>Ascendancy Research</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Browsable (login)</t>
+          <t>Browsable</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>https://experienceapc.com/getting-started</t>
+          <t>https://studies.ascendresearch.com/</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Atkins Research</t>
+          <t>Askable</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Email-only</t>
+          <t>Unclear</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>https://www.atkinsresearch.com/research-participant/respondent-signup/</t>
+          <t>https://www.askable.com/earn/participants</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Become A Thinker</t>
+          <t>ATH Power Consulting</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Browsable</t>
+          <t>Browsable (login)</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>https://becomeathinker.com/upcoming-studies/</t>
+          <t>https://experienceapc.com/getting-started</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>BestMark</t>
+          <t>Atkins Research</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Browsable (login)</t>
+          <t>Email-only</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>https://secure.bestmark.com/public/application/appstart.aspx</t>
+          <t>https://www.atkinsresearch.com/research-participant/respondent-signup/</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Bezel Research</t>
+          <t>Become A Thinker</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Email-only</t>
+          <t>Browsable</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>http://bezelrr.com/</t>
+          <t>https://becomeathinker.com/upcoming-studies/</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Big Bang Recruiting</t>
+          <t>BestMark</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Email-only</t>
+          <t>Browsable (login)</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>https://www.bigbangrecruiting.com/register/</t>
+          <t>https://secure.bestmark.com/public/application/appstart.aspx</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Blink UX</t>
+          <t>Bezel Research</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Unclear</t>
+          <t>Email-only</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>https://participate.blinkux.com/</t>
+          <t>http://bezelrr.com/</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Brightside Research Solutions</t>
+          <t>Big Bang Recruiting</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -783,48 +783,48 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>https://teambrightsider.com/</t>
+          <t>https://www.bigbangrecruiting.com/register/</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Cambridge Focus</t>
+          <t>Blink UX</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Email-only</t>
+          <t>Unclear</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>http://www.participatenewengland.com/</t>
+          <t>https://participate.blinkux.com/</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Cara Casting</t>
+          <t>Brightside Research Solutions</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Browsable</t>
+          <t>Email-only</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>https://jobs.caracasting.com/</t>
+          <t>https://teambrightsider.com/</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>CIC Testing</t>
+          <t>Cambridge Focus</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -834,31 +834,31 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>https://www.cictesting.com/CIC/</t>
+          <t>http://www.participatenewengland.com/</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Citrus Labs</t>
+          <t>Cara Casting</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Email-only</t>
+          <t>Browsable</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>https://www.citruslabs.com/</t>
+          <t>https://jobs.caracasting.com/</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>ClearView Research</t>
+          <t>CEC Surveys</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -868,14 +868,14 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>http://www.clearviewresearch.com/sign-up-now.aspx</t>
+          <t>https://cecsurveys.com/</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Collab Research</t>
+          <t>CIC Testing</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -885,14 +885,14 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>https://www.collab-research.com/</t>
+          <t>https://www.cictesting.com/CIC/</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Compass Research</t>
+          <t>Citrus Labs</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -902,14 +902,14 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>https://compassmarketingresearch.com/sign-up/</t>
+          <t>https://www.citruslabs.com/</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Confide Research</t>
+          <t>ClearView Research</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -919,31 +919,31 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>https://confideresearch.com/Participants/signup</t>
+          <t>http://www.clearviewresearch.com/sign-up-now.aspx</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>ConneXion Research</t>
+          <t>Collab Research</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Browsable</t>
+          <t>Email-only</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>https://jointheconnexion.com/current-projects/</t>
+          <t>https://www.collab-research.com/</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Consumer Viewpoint</t>
+          <t>Compass Research</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -953,14 +953,14 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>https://www.paidforyouropinions.com</t>
+          <t>https://compassmarketingresearch.com/sign-up/</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Contact Design</t>
+          <t>Confide Research</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -970,61 +970,65 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>https://yourcontacthub.com/</t>
+          <t>https://confideresearch.com/Participants/signup</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Contract Testing</t>
+          <t>ConneXion Research</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Email-only</t>
+          <t>Browsable</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>https://connect.contracttesting.com/ctimvc/Account/Register</t>
+          <t>https://jointheconnexion.com/current-projects/</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Core</t>
+          <t>Consumer Viewpoint</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Unclear</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr"/>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>https://www.paidforyouropinions.com</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Curion</t>
+          <t>Contact Design</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Browsable (login)</t>
+          <t>Email-only</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>https://curionpanelist.com/portal/default</t>
+          <t>https://yourcontacthub.com/</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Cypher Research</t>
+          <t>Contract Testing</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1034,48 +1038,44 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>https://cypherresearch.com/intranet/respondent_sign_up.php</t>
+          <t>https://connect.contracttesting.com/ctimvc/Account/Register</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Daisy Mae Research</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Browsable</t>
-        </is>
-      </c>
-      <c r="C37" s="2" t="inlineStr">
-        <is>
-          <t>https://daisymaeresearch.com/projects/</t>
-        </is>
-      </c>
+          <t>Unclear</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Decision Point Research</t>
+          <t>Curion</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Email-only</t>
+          <t>Browsable (login)</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>https://www.decisionpointresearch.ca</t>
+          <t>https://curionpanelist.com/portal/default</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Design Science</t>
+          <t>Cypher Research</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1085,48 +1085,48 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>https://dscience.com/signup</t>
+          <t>https://cypherresearch.com/intranet/respondent_sign_up.php</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Drive Research</t>
+          <t>Daisy Mae Research</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Email-only</t>
+          <t>Browsable</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>https://www.driveresearch.com/participate/</t>
+          <t>https://daisymaeresearch.com/projects/</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>dscout</t>
+          <t>Decision Point Research</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Browsable (mobile app)</t>
+          <t>Email-only</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>https://dscout.com</t>
+          <t>https://www.decisionpointresearch.ca</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Elliott Benson</t>
+          <t>Design Science</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1136,48 +1136,48 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>https://www.elliottbenson.com/participate/</t>
+          <t>https://dscience.com/signup</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>End to End Research</t>
+          <t>Drive Research</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Unclear</t>
+          <t>Email-only</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>https://www.endtoenduserresearch.com/participate.html</t>
+          <t>https://www.driveresearch.com/participate/</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Engage In Depth</t>
+          <t>dscout</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Email-only</t>
+          <t>Browsable (mobile app)</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>https://engageindepth.com/participate/</t>
+          <t>https://dscout.com</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Ethical Mind</t>
+          <t>Elliott Benson</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1187,65 +1187,65 @@
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>https://ethicalmind.org/</t>
+          <t>https://www.elliottbenson.com/participate/</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>FF Focus Group</t>
+          <t>EmCee Research</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Browsable</t>
+          <t>Email-only</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>https://www.fffocusgroup.com/current-projects/</t>
+          <t>https://emceeresearch.com/</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Field Agent / Storesight</t>
+          <t>End to End Research</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Browsable (login)</t>
+          <t>Unclear</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>https://app.fieldagent.net/</t>
+          <t>https://www.endtoenduserresearch.com/participate.html</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Field Voices</t>
+          <t>Engage In Depth</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Browsable</t>
+          <t>Email-only</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>https://fieldvoices.com/current_studies</t>
+          <t>https://engageindepth.com/participate/</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Fieldwork</t>
+          <t>Ethical Mind</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1255,65 +1255,65 @@
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>https://www.fieldwork.com</t>
+          <t>https://ethicalmind.org/</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>First Court Jurors</t>
+          <t>FF Focus Group</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Email-only</t>
+          <t>Browsable</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>https://www.firstcourt.com/jury-recruiting</t>
+          <t>https://www.fffocusgroup.com/current-projects/</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Fleischman Field Research</t>
+          <t>Field Agent / Storesight</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Email-only</t>
+          <t>Browsable (login)</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>http://www.ffrsf.com/</t>
+          <t>https://app.fieldagent.net/</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Focus &amp; Testing</t>
+          <t>Field Voices</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Email-only</t>
+          <t>Browsable</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>https://research.focusandtesting.com/</t>
+          <t>https://fieldvoices.com/current_studies</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>focus 99</t>
+          <t>Fieldwork</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -1323,14 +1323,14 @@
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>https://www.focus99.com/sub/</t>
+          <t>https://www.fieldwork.com</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Focus Corner</t>
+          <t>First Court Jurors</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1340,14 +1340,14 @@
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>https://focuscorner.net/</t>
+          <t>https://www.firstcourt.com/jury-recruiting</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Focus Crossroads</t>
+          <t>Fleischman Field Research</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -1357,14 +1357,14 @@
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>https://focuscrossroads.org/research-network/join-consumer/</t>
+          <t>http://www.ffrsf.com/</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Focus Group Connection</t>
+          <t>Focus &amp; Testing</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1374,48 +1374,48 @@
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>https://www.focusgroupconnection.com/participate/</t>
+          <t>https://research.focusandtesting.com/</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Focus Group Panel</t>
+          <t>focus 99</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Browsable</t>
+          <t>Email-only</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>https://focusgrouppanel.com/research-category/focus-group/</t>
+          <t>https://www.focus99.com/sub/</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Focus Insite</t>
+          <t>Focus Corner</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Unclear</t>
+          <t>Email-only</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>https://linktr.ee/focus_insite</t>
+          <t>https://focuscorner.net/</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Focus Pulse</t>
+          <t>Focus Crossroads</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -1425,31 +1425,31 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>https://focuspulseresearch.co.uk/</t>
+          <t>https://focuscrossroads.org/research-network/join-consumer/</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Focus Room</t>
+          <t>Focus Group Connection</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Browsable</t>
+          <t>Email-only</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>https://focusroom.com/active-studies/</t>
+          <t>https://www.focusgroupconnection.com/participate/</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Focuscope</t>
+          <t>Focus Group Finder</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -1459,48 +1459,48 @@
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>https://www.focuscope.com/join-our-community/</t>
+          <t>https://focusgroups.org/</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Funds for Focus</t>
+          <t>Focus Group Panel</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Unclear</t>
+          <t>Browsable</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>https://fundsforfocus.com/</t>
+          <t>https://focusgrouppanel.com/research-category/focus-group/</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Galloway Research</t>
+          <t>Focus Insite</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Browsable</t>
+          <t>Unclear</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>https://www.questionspace.net/category/upcoming-studies/</t>
+          <t>https://linktr.ee/focus_insite</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Georgetown University (GRVP)</t>
+          <t>Focus Pulse</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1510,14 +1510,14 @@
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>https://grvp.georgetown.edu/</t>
+          <t>https://focuspulseresearch.co.uk/</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Good Gamer Group</t>
+          <t>Focus Room</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1527,14 +1527,14 @@
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>https://goodgamergroup.com/available-studies/</t>
+          <t>https://focusroom.com/active-studies/</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Griot Recruit</t>
+          <t>Focuscope</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1544,82 +1544,82 @@
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>https://www.griotrecruit.co/</t>
+          <t>https://www.focuscope.com/join-our-community/</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Hagen Sinclair Research Recruiting</t>
+          <t>Funds for Focus</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Email-only</t>
+          <t>Unclear</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>https://hagensinclair.com/paid-research-studies-2/</t>
+          <t>https://fundsforfocus.com/</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Horizon Group</t>
+          <t>Galloway Research</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Email-only</t>
+          <t>Browsable</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>https://www.horizongroupiowa.com/join-our-panel/</t>
+          <t>https://www.questionspace.net/category/upcoming-studies/</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>IDEO Design Research</t>
+          <t>Georgetown University (GRVP)</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Browsable</t>
+          <t>Email-only</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>https://designresearch.ideo.com/opportunities</t>
+          <t>https://grvp.georgetown.edu/</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Insight Recruit</t>
+          <t>Good Gamer Group</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Email-only</t>
+          <t>Browsable</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>https://insightrecruit.com/join-our-panel/</t>
+          <t>https://goodgamergroup.com/available-studies/</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Intact Qualitative Research</t>
+          <t>Griot Recruit</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -1629,65 +1629,65 @@
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>https://www.iqrsf.com/participant-intake-form</t>
+          <t>https://www.griotrecruit.co/</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>ISG (Information Specialists Group)</t>
+          <t>Hagen Sinclair Research Recruiting</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Unclear</t>
+          <t>Email-only</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>http://www.isgpanel.com/</t>
+          <t>https://hagensinclair.com/paid-research-studies-2/</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Ivy Exec</t>
+          <t>Horizon Group</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Browsable (login)</t>
+          <t>Email-only</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>https://ivyexec.com/jobs-and-research-studies-search?type=study</t>
+          <t>https://www.horizongroupiowa.com/join-our-panel/</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Jackson Associates</t>
+          <t>IDEO Design Research</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Browsable (login)</t>
+          <t>Browsable</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>https://research.jacksonassociates.com/</t>
+          <t>https://designresearch.ideo.com/opportunities</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>JC Research Partners</t>
+          <t>Insight Recruit</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -1697,48 +1697,48 @@
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>https://jcresearchpartners.com/</t>
+          <t>https://insightrecruit.com/join-our-panel/</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>JJA Research</t>
+          <t>Intact Qualitative Research</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Browsable</t>
+          <t>Email-only</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>https://jjarecruiting.com/?post_type=project</t>
+          <t>https://www.iqrsf.com/participant-intake-form</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>KSS International</t>
+          <t>ISG (Information Specialists Group)</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Browsable (login)</t>
+          <t>Unclear</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>http://kernscheduling.com/</t>
+          <t>http://www.isgpanel.com/</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>L&amp;E Research</t>
+          <t>Ivy Exec</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -1748,99 +1748,99 @@
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>https://www.leopinions.com/</t>
+          <t>https://ivyexec.com/jobs-and-research-studies-search?type=study</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Leede Research</t>
+          <t>Jackson Associates</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Browsable</t>
+          <t>Browsable (login)</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>https://leedemn.com/join-our-database/available-studies/</t>
+          <t>https://research.jacksonassociates.com/</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Lees Focus</t>
+          <t>JC Research Partners</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Browsable</t>
+          <t>Email-only</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>https://leesfocusgroups.com/</t>
+          <t>https://jcresearchpartners.com/</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Limelight by Shugoll</t>
+          <t>JJA Research</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Email-only</t>
+          <t>Browsable</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>https://limelightbyshugoll.com/get-paid-for-your-opinion/</t>
+          <t>https://jjarecruiting.com/?post_type=project</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Local Focus Group</t>
+          <t>KSS International</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Email-only</t>
+          <t>Browsable (login)</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>https://www.localfocusgroup.com/</t>
+          <t>http://kernscheduling.com/</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>MacConnell Research</t>
+          <t>L&amp;E Research</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Unclear</t>
+          <t>Browsable (login)</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>http://www.macconnellresearch.com/</t>
+          <t>https://www.leopinions.com/</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Market-Ease (Market Eaze)</t>
+          <t>Leede Research</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -1850,31 +1850,31 @@
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>https://www.market-ease.com/about-the-respondent-hub</t>
+          <t>https://leedemn.com/join-our-database/available-studies/</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>MarketForce</t>
+          <t>Lees Focus</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Browsable (login)</t>
+          <t>Browsable</t>
         </is>
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>https://shopper.marketforce.com/</t>
+          <t>https://leesfocusgroups.com/</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Mars Research</t>
+          <t>Limelight by Shugoll</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -1884,14 +1884,14 @@
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>https://joinmarsresearch.com/</t>
+          <t>https://limelightbyshugoll.com/get-paid-for-your-opinion/</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>McCormick Group</t>
+          <t>Local Focus Group</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -1901,82 +1901,82 @@
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>http://mccormick-group.com/market-research.html</t>
+          <t>https://www.localfocusgroup.com/</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Mediabarn Research</t>
+          <t>MacConnell Research</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Browsable</t>
+          <t>Unclear</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>https://www.mediabarnresearch.com/currentstudies/</t>
+          <t>http://www.macconnellresearch.com/</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>MeThinks</t>
+          <t>Market-Ease (Market Eaze)</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Browsable (login)</t>
+          <t>Browsable</t>
         </is>
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>https://www.methinks.io/thinker</t>
+          <t>https://www.market-ease.com/about-the-respondent-hub</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>MForce Research</t>
+          <t>MarketForce</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Email-only</t>
+          <t>Browsable (login)</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>http://www.mforceresearch.com/</t>
+          <t>https://shopper.marketforce.com/</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Mindswarms</t>
+          <t>Mars Research</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Browsable (login)</t>
+          <t>Email-only</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>https://app.mindswarms.com/sign_in</t>
+          <t>https://joinmarsresearch.com/</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Moore Opinions</t>
+          <t>McCormick Group</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -1986,48 +1986,48 @@
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>http://mooreopinions.com/</t>
+          <t>http://mccormick-group.com/market-research.html</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Moore Research Services</t>
+          <t>Mediabarn Research</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Email-only</t>
+          <t>Browsable</t>
         </is>
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>https://www.moore-research.com/join-a-panel/</t>
+          <t>https://www.mediabarnresearch.com/currentstudies/</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Murray Hill National</t>
+          <t>MeThinks</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Unclear</t>
+          <t>Browsable (login)</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>https://panels.murrayhillnational.com/Portal/Default</t>
+          <t>https://www.methinks.io/thinker</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>MVG Recruiting</t>
+          <t>MForce Research</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2037,65 +2037,65 @@
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>https://mvgrecruiting.com/sign-up</t>
+          <t>http://www.mforceresearch.com/</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>N.C. Litigation &amp; Jury Research Group</t>
+          <t>Mindswarms</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Email-only</t>
+          <t>Browsable (login)</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>https://ncfocusgroups.com/</t>
+          <t>https://app.mindswarms.com/sign_in</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Nashville Research Group</t>
+          <t>Moore Opinions</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Browsable</t>
+          <t>Email-only</t>
         </is>
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>https://www.nashvilleresearch.com/current-research-projects</t>
+          <t>http://mooreopinions.com/</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Nationwide Research Recruiters</t>
+          <t>Moore Research Services</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Browsable</t>
+          <t>Email-only</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>https://www.nwrrs.com/focus-group-calendar.html</t>
+          <t>https://www.moore-research.com/join-a-panel/</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>NDR (National Data Research)</t>
+          <t>Murray Hill National</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2105,14 +2105,14 @@
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>http://www.national-data.net/</t>
+          <t>https://panels.murrayhillnational.com/Portal/Default</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Nelson Recruiting</t>
+          <t>MVG Recruiting</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -2122,14 +2122,14 @@
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>https://nelsonrecruiting.com</t>
+          <t>https://mvgrecruiting.com/sign-up</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>New England Focus Group</t>
+          <t>N.C. Litigation &amp; Jury Research Group</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -2139,61 +2139,65 @@
       </c>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>https://www.newenglandfocusgroup.com/register.html</t>
+          <t>https://ncfocusgroups.com/</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Newton (ambiguous)</t>
+          <t>Nashville Research Group</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Unclear</t>
-        </is>
-      </c>
-      <c r="C102" t="inlineStr"/>
+          <t>Browsable</t>
+        </is>
+      </c>
+      <c r="C102" s="2" t="inlineStr">
+        <is>
+          <t>https://www.nashvilleresearch.com/current-research-projects</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Newton Marketing Network</t>
+          <t>Nationwide Research Recruiters</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Email-only</t>
+          <t>Browsable</t>
         </is>
       </c>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>https://newtonmarketingnetwork.com/participants/</t>
+          <t>https://www.nwrrs.com/focus-group-calendar.html</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Nichols Research</t>
+          <t>NDR (National Data Research)</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Email-only</t>
+          <t>Unclear</t>
         </is>
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>https://nicholsresearch.com/registration-form/</t>
+          <t>http://www.national-data.net/</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>NYC Focal (The Diamond Lists)</t>
+          <t>Nelson Recruiting</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -2203,82 +2207,78 @@
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>https://thediamondlists.com/join-the-list/</t>
+          <t>https://nelsonrecruiting.com</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Olympic National Research</t>
+          <t>New England Focus Group</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Unclear</t>
+          <t>Email-only</t>
         </is>
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>https://olympicnationalprojects.com/</t>
+          <t>https://www.newenglandfocusgroup.com/register.html</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Online Verdict</t>
+          <t>Newton (ambiguous)</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Email-only</t>
-        </is>
-      </c>
-      <c r="C107" s="2" t="inlineStr">
-        <is>
-          <t>https://www.onlineverdict.com/jurors/signup/</t>
-        </is>
-      </c>
+          <t>Unclear</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Opinions by Sync</t>
+          <t>Newton Marketing Network</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Browsable</t>
+          <t>Email-only</t>
         </is>
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>https://community.opinionsbysync.com/s/Jobsite</t>
+          <t>https://newtonmarketingnetwork.com/participants/</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Opinions for Cash</t>
+          <t>Nichols Research</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Unclear</t>
+          <t>Email-only</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
         <is>
-          <t>https://opinionsforcash.com/</t>
+          <t>https://nicholsresearch.com/registration-form/</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Opinions Link</t>
+          <t>NYC Focal (The Diamond Lists)</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -2288,320 +2288,320 @@
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>https://www.opinionslink.com</t>
+          <t>https://thediamondlists.com/join-the-list/</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Opinions LTD</t>
+          <t>Olympic National Research</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Email-only</t>
+          <t>Unclear</t>
         </is>
       </c>
       <c r="C111" s="2" t="inlineStr">
         <is>
-          <t>https://www.opinionsltd.com/participate/</t>
+          <t>https://olympicnationalprojects.com/</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Orman Guidance</t>
+          <t>Online Verdict</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Browsable</t>
+          <t>Email-only</t>
         </is>
       </c>
       <c r="C112" s="2" t="inlineStr">
         <is>
-          <t>https://ormanguidance.com/participate/projects/</t>
+          <t>https://www.onlineverdict.com/jurors/signup/</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>People for Research</t>
+          <t>Opinions by Sync</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Browsable (login)</t>
+          <t>Browsable</t>
         </is>
       </c>
       <c r="C113" s="2" t="inlineStr">
         <is>
-          <t>https://www.peopleforresearch.co.uk/participant/opportunities</t>
+          <t>https://community.opinionsbysync.com/s/Jobsite</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Portable Insights</t>
+          <t>Opinions for Cash</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Email-only</t>
+          <t>Unclear</t>
         </is>
       </c>
       <c r="C114" s="2" t="inlineStr">
         <is>
-          <t>https://portableinsights.com/join-our-panel</t>
+          <t>https://opinionsforcash.com/</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Pragmatic Research</t>
+          <t>Opinions Link</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Unclear</t>
+          <t>Email-only</t>
         </is>
       </c>
       <c r="C115" s="2" t="inlineStr">
         <is>
-          <t>http://www.pragmatic-research.com/</t>
+          <t>https://www.opinionslink.com</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>PRC</t>
+          <t>Opinions LTD</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Browsable</t>
+          <t>Email-only</t>
         </is>
       </c>
       <c r="C116" s="2" t="inlineStr">
         <is>
-          <t>https://www.prcmarketresearch.com/upcomingprojects</t>
+          <t>https://www.opinionsltd.com/participate/</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Precision Research</t>
+          <t>Orman Guidance</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Email-only</t>
+          <t>Browsable</t>
         </is>
       </c>
       <c r="C117" s="2" t="inlineStr">
         <is>
-          <t>https://www.opinionwizard.com/</t>
+          <t>https://ormanguidance.com/participate/projects/</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Prepare to Persuade</t>
+          <t>People for Research</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Unclear</t>
+          <t>Browsable (login)</t>
         </is>
       </c>
       <c r="C118" s="2" t="inlineStr">
         <is>
-          <t>https://www.preparetopersuade.com</t>
+          <t>https://www.peopleforresearch.co.uk/participant/opportunities</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Private Jury</t>
+          <t>Portable Insights</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Browsable</t>
+          <t>Email-only</t>
         </is>
       </c>
       <c r="C119" s="2" t="inlineStr">
         <is>
-          <t>https://www.privatejury.com/</t>
+          <t>https://portableinsights.com/join-our-panel</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>Probe Market Research</t>
+          <t>Pragmatic Research</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Browsable</t>
+          <t>Unclear</t>
         </is>
       </c>
       <c r="C120" s="2" t="inlineStr">
         <is>
-          <t>https://www.probemarket.com/available-studies/</t>
+          <t>http://www.pragmatic-research.com/</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Product Tube</t>
+          <t>PRC</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Email-only</t>
+          <t>Browsable</t>
         </is>
       </c>
       <c r="C121" s="2" t="inlineStr">
         <is>
-          <t>https://web.producttube.com/signup</t>
+          <t>https://www.prcmarketresearch.com/upcomingprojects</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>Prolific</t>
+          <t>Precision Research</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>Browsable (login)</t>
+          <t>Email-only</t>
         </is>
       </c>
       <c r="C122" s="2" t="inlineStr">
         <is>
-          <t>https://app.prolific.com/</t>
+          <t>https://www.opinionwizard.com/</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>PVR Research</t>
+          <t>Prepare to Persuade</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>Email-only</t>
+          <t>Unclear</t>
         </is>
       </c>
       <c r="C123" s="2" t="inlineStr">
         <is>
-          <t>http://www.pvr-research.com/</t>
+          <t>https://www.preparetopersuade.com</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>Q-Insights</t>
+          <t>Private Jury</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>Email-only</t>
+          <t>Browsable</t>
         </is>
       </c>
       <c r="C124" s="2" t="inlineStr">
         <is>
-          <t>https://q-insights.com/</t>
+          <t>https://www.privatejury.com/</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>Qual Recruit</t>
+          <t>Probe Market Research</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>Email-only</t>
+          <t>Browsable</t>
         </is>
       </c>
       <c r="C125" s="2" t="inlineStr">
         <is>
-          <t>https://www.qualrecruit.com/become-a-participant</t>
+          <t>https://www.probemarket.com/available-studies/</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Rare Patient Voice</t>
+          <t>Product Tube</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>Browsable</t>
+          <t>Email-only</t>
         </is>
       </c>
       <c r="C126" s="2" t="inlineStr">
         <is>
-          <t>https://rarepatientvoice.com/for-patients/study-opportunities/</t>
+          <t>https://web.producttube.com/signup</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>Real Focus Group</t>
+          <t>Prolific</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>Browsable</t>
+          <t>Browsable (login)</t>
         </is>
       </c>
       <c r="C127" s="2" t="inlineStr">
         <is>
-          <t>https://realfocusgroup.com/upcoming/</t>
+          <t>https://app.prolific.com/</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>Reckner</t>
+          <t>Pulse Labs</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>Email-only</t>
+          <t>Browsable (login)</t>
         </is>
       </c>
       <c r="C128" s="2" t="inlineStr">
         <is>
-          <t>https://www.reckner.com</t>
+          <t>https://app.pulselabs.ai/</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>Recruit and Field</t>
+          <t>PVR Research</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -2611,31 +2611,31 @@
       </c>
       <c r="C129" s="2" t="inlineStr">
         <is>
-          <t>https://www.recruitandfield.com/register-as-a-participant</t>
+          <t>http://www.pvr-research.com/</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>Research America</t>
+          <t>Q-Insights</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>Unclear</t>
+          <t>Email-only</t>
         </is>
       </c>
       <c r="C130" s="2" t="inlineStr">
         <is>
-          <t>https://researchamericainc.net/</t>
+          <t>https://q-insights.com/</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>Research Outloud</t>
+          <t>Qual Recruit</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -2645,48 +2645,48 @@
       </c>
       <c r="C131" s="2" t="inlineStr">
         <is>
-          <t>https://researchoutloud.com/</t>
+          <t>https://www.qualrecruit.com/become-a-participant</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>Respondent</t>
+          <t>Rare Patient Voice</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>Browsable (login)</t>
+          <t>Browsable</t>
         </is>
       </c>
       <c r="C132" s="2" t="inlineStr">
         <is>
-          <t>https://app.respondent.io/respondents/v2/projects/browse</t>
+          <t>https://rarepatientvoice.com/for-patients/study-opportunities/</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>Ridgeline Recruiting</t>
+          <t>Real Focus Group</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>Email-only</t>
+          <t>Browsable</t>
         </is>
       </c>
       <c r="C133" s="2" t="inlineStr">
         <is>
-          <t>https://ridgelinerecruiting.com/</t>
+          <t>https://realfocusgroup.com/upcoming/</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>Round2Research</t>
+          <t>Reckner</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -2696,14 +2696,14 @@
       </c>
       <c r="C134" s="2" t="inlineStr">
         <is>
-          <t>https://round2research.com/</t>
+          <t>https://www.reckner.com</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>RRU Research</t>
+          <t>Recruit and Field</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -2713,48 +2713,48 @@
       </c>
       <c r="C135" s="2" t="inlineStr">
         <is>
-          <t>https://focuspocussoftware.net/WP_RRU/Register</t>
+          <t>https://www.recruitandfield.com/register-as-a-participant</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>SAGO (Schlesinger / Focus Pointe Global)</t>
+          <t>Research America</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>Browsable (login)</t>
+          <t>Unclear</t>
         </is>
       </c>
       <c r="C136" s="2" t="inlineStr">
         <is>
-          <t>https://www.focusgroup.com/</t>
+          <t>https://researchamericainc.net/</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>Savvy Cooperative</t>
+          <t>Research Outloud</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>Browsable (login)</t>
+          <t>Email-only</t>
         </is>
       </c>
       <c r="C137" s="2" t="inlineStr">
         <is>
-          <t>https://apply.savvy.coop/</t>
+          <t>https://researchoutloud.com/</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>Secret Shopper</t>
+          <t>Respondent</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -2764,14 +2764,14 @@
       </c>
       <c r="C138" s="2" t="inlineStr">
         <is>
-          <t>https://www.secretshopper.com/shoppers/shoppers</t>
+          <t>https://app.respondent.io/respondents/v2/projects/browse</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>SIS Research</t>
+          <t>Ridgeline Recruiting</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
@@ -2781,14 +2781,14 @@
       </c>
       <c r="C139" s="2" t="inlineStr">
         <is>
-          <t>https://participate.sisinternational.com/Portal/Default</t>
+          <t>https://ridgelinerecruiting.com/</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>Spotlight Research</t>
+          <t>Round2Research</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
@@ -2798,116 +2798,116 @@
       </c>
       <c r="C140" s="2" t="inlineStr">
         <is>
-          <t>https://spotlightmarketresearch.com/join-our-audience/</t>
+          <t>https://round2research.com/</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>Take Part in Research</t>
+          <t>RRU Research</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>Browsable</t>
+          <t>Email-only</t>
         </is>
       </c>
       <c r="C141" s="2" t="inlineStr">
         <is>
-          <t>https://takepartinresearch.co.uk/current-projects/</t>
+          <t>https://focuspocussoftware.net/WP_RRU/Register</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>Talking Heads</t>
+          <t>SAGO (Schlesinger / Focus Pointe Global)</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>Email-only</t>
+          <t>Browsable (login)</t>
         </is>
       </c>
       <c r="C142" s="2" t="inlineStr">
         <is>
-          <t>http://register.talkingheadsstudio.com/</t>
+          <t>https://www.focusgroup.com/</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>Taylor Research</t>
+          <t>Savvy Cooperative</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>Unclear</t>
+          <t>Browsable (login)</t>
         </is>
       </c>
       <c r="C143" s="2" t="inlineStr">
         <is>
-          <t>https://studies.taylorresearch.com/</t>
+          <t>https://apply.savvy.coop/</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>The Heard</t>
+          <t>Secret Shopper</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>Browsable</t>
+          <t>Browsable (login)</t>
         </is>
       </c>
       <c r="C144" s="2" t="inlineStr">
         <is>
-          <t>https://www.betheheard.com</t>
+          <t>https://www.secretshopper.com/shoppers/shoppers</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>The Insighters</t>
+          <t>SIS Research</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>Browsable</t>
+          <t>Email-only</t>
         </is>
       </c>
       <c r="C145" s="2" t="inlineStr">
         <is>
-          <t>https://theinsighters.com/public-opportunities</t>
+          <t>https://participate.sisinternational.com/Portal/Default</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>The Social Question</t>
+          <t>Spotlight Research</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>Browsable</t>
+          <t>Email-only</t>
         </is>
       </c>
       <c r="C146" s="2" t="inlineStr">
         <is>
-          <t>https://www.the-socialq.com/open-studies</t>
+          <t>https://spotlightmarketresearch.com/join-our-audience/</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>Theoretics</t>
+          <t>Take Part in Research</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -2917,31 +2917,31 @@
       </c>
       <c r="C147" s="2" t="inlineStr">
         <is>
-          <t>https://www.theoretics.co/current-projects</t>
+          <t>https://takepartinresearch.co.uk/current-projects/</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>TrendSource</t>
+          <t>Talking Heads</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>Browsable (login)</t>
+          <t>Email-only</t>
         </is>
       </c>
       <c r="C148" s="2" t="inlineStr">
         <is>
-          <t>https://www.thesourceagents.com/</t>
+          <t>http://register.talkingheadsstudio.com/</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>Truscott Research</t>
+          <t>Taylor Research</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -2951,65 +2951,65 @@
       </c>
       <c r="C149" s="2" t="inlineStr">
         <is>
-          <t>https://app.truscottresearch.com/register</t>
+          <t>https://studies.taylorresearch.com/</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>Ubinsights</t>
+          <t>TELUS Digital (research)</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>Email-only</t>
+          <t>Unclear</t>
         </is>
       </c>
       <c r="C150" s="2" t="inlineStr">
         <is>
-          <t>https://ubinsights.com/</t>
+          <t>https://www.telusinternational.com/</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>Uncover Research</t>
+          <t>The Heard</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>Email-only</t>
+          <t>Browsable</t>
         </is>
       </c>
       <c r="C151" s="2" t="inlineStr">
         <is>
-          <t>https://www.uncoverresearch.com/participate</t>
+          <t>https://www.betheheard.com</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>User Insight</t>
+          <t>The Insighters</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>Email-only</t>
+          <t>Browsable</t>
         </is>
       </c>
       <c r="C152" s="2" t="inlineStr">
         <is>
-          <t>https://www.shareyourinsights.com/</t>
+          <t>https://theinsighters.com/public-opportunities</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>User Interviews</t>
+          <t>The Social Question</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -3019,82 +3019,82 @@
       </c>
       <c r="C153" s="2" t="inlineStr">
         <is>
-          <t>https://www.userinterviews.com/studies</t>
+          <t>https://www.the-socialq.com/open-studies</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>User Research International</t>
+          <t>Theoretics</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>Browsable (login)</t>
+          <t>Browsable</t>
         </is>
       </c>
       <c r="C154" s="2" t="inlineStr">
         <is>
-          <t>https://app.uriux.com/studies</t>
+          <t>https://www.theoretics.co/current-projects</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>uTest</t>
+          <t>Thurs Recruiting</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>Browsable (login)</t>
+          <t>Email-only</t>
         </is>
       </c>
       <c r="C155" s="2" t="inlineStr">
         <is>
-          <t>https://www.utest.com/projects</t>
+          <t>https://thursrecruiting.com/</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>Videochat Network</t>
+          <t>TrendSource</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>Email-only</t>
+          <t>Browsable (login)</t>
         </is>
       </c>
       <c r="C156" s="2" t="inlineStr">
         <is>
-          <t>https://www.videochatnetwork.net/sign-up/</t>
+          <t>https://www.thesourceagents.com/</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>View-Finders</t>
+          <t>Truscott Research</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>Email-only</t>
+          <t>Unclear</t>
         </is>
       </c>
       <c r="C157" s="2" t="inlineStr">
         <is>
-          <t>https://www.view-finders.net/participant-registration-2/</t>
+          <t>https://app.truscottresearch.com/register</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>WAC Research</t>
+          <t>Ubinsights</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
@@ -3104,14 +3104,14 @@
       </c>
       <c r="C158" s="2" t="inlineStr">
         <is>
-          <t>https://wacresearch.com/data.html</t>
+          <t>https://ubinsights.com/</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>Watch Me Think</t>
+          <t>Uncover Research</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -3121,14 +3121,14 @@
       </c>
       <c r="C159" s="2" t="inlineStr">
         <is>
-          <t>https://watchmethink.com/contribute</t>
+          <t>https://www.uncoverresearch.com/participate</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>Watchlab</t>
+          <t>User Insight</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -3138,54 +3138,224 @@
       </c>
       <c r="C160" s="2" t="inlineStr">
         <is>
-          <t>https://watchlab.com/sign-up/</t>
+          <t>https://www.shareyourinsights.com/</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>When Opinions Meet</t>
+          <t>User Interviews</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>Unclear</t>
-        </is>
-      </c>
-      <c r="C161" t="inlineStr"/>
+          <t>Browsable</t>
+        </is>
+      </c>
+      <c r="C161" s="2" t="inlineStr">
+        <is>
+          <t>https://www.userinterviews.com/studies</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>Wilkins Research Services</t>
+          <t>User Research International</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>Email-only</t>
+          <t>Browsable (login)</t>
         </is>
       </c>
       <c r="C162" s="2" t="inlineStr">
         <is>
-          <t>https://wilkinsresearch.net/join-our-panel/</t>
+          <t>https://app.uriux.com/studies</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
+          <t>uTest</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>Browsable (login)</t>
+        </is>
+      </c>
+      <c r="C163" s="2" t="inlineStr">
+        <is>
+          <t>https://www.utest.com/projects</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>VGM (playtests)</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C164" s="2" t="inlineStr">
+        <is>
+          <t>https://vgm.co/</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>Videochat Network</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C165" s="2" t="inlineStr">
+        <is>
+          <t>https://www.videochatnetwork.net/sign-up/</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>View-Finders</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C166" s="2" t="inlineStr">
+        <is>
+          <t>https://www.view-finders.net/participant-registration-2/</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>WAC Research</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C167" s="2" t="inlineStr">
+        <is>
+          <t>https://wacresearch.com/data.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>Watch Me Think</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C168" s="2" t="inlineStr">
+        <is>
+          <t>https://watchmethink.com/contribute</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>Watchlab</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C169" s="2" t="inlineStr">
+        <is>
+          <t>https://watchlab.com/sign-up/</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>When Opinions Meet</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>Unclear</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr"/>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>Wilkins Research Services</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C171" s="2" t="inlineStr">
+        <is>
+          <t>https://wilkinsresearch.net/join-our-panel/</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
           <t>Winn Winn Research</t>
         </is>
       </c>
-      <c r="B163" t="inlineStr">
-        <is>
-          <t>Email-only</t>
-        </is>
-      </c>
-      <c r="C163" s="2" t="inlineStr">
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>Email-only</t>
+        </is>
+      </c>
+      <c r="C172" s="2" t="inlineStr">
         <is>
           <t>https://winnwinn.com/new/public/register</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>Wynter</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>Unclear</t>
+        </is>
+      </c>
+      <c r="C173" s="2" t="inlineStr">
+        <is>
+          <t>https://wynter.com/panel</t>
         </is>
       </c>
     </row>
@@ -3223,9 +3393,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId30"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId31"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C33" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C35" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C36" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C37" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C34" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C35" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C36" r:id="rId35"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C38" r:id="rId36"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C39" r:id="rId37"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C40" r:id="rId38"/>
@@ -3290,11 +3460,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C99" r:id="rId97"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C100" r:id="rId98"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C101" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C103" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C104" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C105" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C106" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C107" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C102" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C103" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C104" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C105" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C106" r:id="rId104"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C108" r:id="rId105"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C109" r:id="rId106"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C110" r:id="rId107"/>
@@ -3348,8 +3518,18 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C158" r:id="rId155"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C159" r:id="rId156"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C160" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C162" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C163" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C161" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C162" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C163" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C164" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C165" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C166" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C167" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C168" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C169" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C171" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C172" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C173" r:id="rId169"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Remove Prolific from catalog
</commit_message>
<xml_diff>
--- a/docs/recruiters.xlsx
+++ b/docs/recruiters.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C172"/>
+  <dimension ref="A1:C171"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -1130,7 +1130,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Prolific</t>
+          <t>Pulse Labs</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1140,14 +1140,14 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>https://app.prolific.com/</t>
+          <t>https://www.pulselabs.ai/</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Pulse Labs</t>
+          <t>Respondent</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1157,14 +1157,14 @@
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>https://www.pulselabs.ai/</t>
+          <t>https://app.respondent.io/respondents/v2/projects/browse</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Respondent</t>
+          <t>SAGO (Schlesinger / Focus Pointe Global)</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1174,14 +1174,14 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>https://app.respondent.io/respondents/v2/projects/browse</t>
+          <t>https://www.focusgroup.com/</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>SAGO (Schlesinger / Focus Pointe Global)</t>
+          <t>Savvy Cooperative</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1191,14 +1191,14 @@
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>https://www.focusgroup.com/</t>
+          <t>https://apply.savvy.coop/</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Savvy Cooperative</t>
+          <t>Secret Shopper</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1208,14 +1208,14 @@
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>https://apply.savvy.coop/</t>
+          <t>https://www.secretshopper.com/shoppers/shoppers</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Secret Shopper</t>
+          <t>TrendSource</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1225,14 +1225,14 @@
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>https://www.secretshopper.com/shoppers/shoppers</t>
+          <t>https://www.thesourceagents.com/</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>TrendSource</t>
+          <t>User Research International</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1242,14 +1242,14 @@
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>https://www.thesourceagents.com/</t>
+          <t>https://app.uriux.com/studies</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>User Research International</t>
+          <t>uTest</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1259,14 +1259,14 @@
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>https://app.uriux.com/studies</t>
+          <t>https://www.utest.com/projects</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>uTest</t>
+          <t>Isecretshop</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1276,14 +1276,14 @@
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>https://www.utest.com/projects</t>
+          <t>https://isecretshop.com/</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Isecretshop</t>
+          <t>10K Voices</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1293,31 +1293,31 @@
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>https://isecretshop.com/</t>
+          <t>https://community.10kvoices.com</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>10K Voices</t>
+          <t>Accelerant Research</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Browsable</t>
+          <t>Email-only</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>https://community.10kvoices.com</t>
+          <t>https://www.accelerantresearch.com/availableresearch</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Accelerant Research</t>
+          <t>Ascendancy Research</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -1327,14 +1327,14 @@
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>https://www.accelerantresearch.com/availableresearch</t>
+          <t>https://www.ascendresearch.com/getpaid</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Ascendancy Research</t>
+          <t>Cara Casting</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1344,14 +1344,14 @@
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>https://www.ascendresearch.com/getpaid</t>
+          <t>https://jobs.caracasting.com/</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Cara Casting</t>
+          <t>FF Focus Group</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -1361,14 +1361,14 @@
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>https://jobs.caracasting.com/</t>
+          <t>https://www.fffocusgroup.com/current-projects/</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>FF Focus Group</t>
+          <t>Field Voices</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1378,14 +1378,14 @@
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>https://www.fffocusgroup.com/current-projects/</t>
+          <t>https://fieldvoices.com/current_studies</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Field Voices</t>
+          <t>Galloway Research</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -1395,14 +1395,14 @@
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>https://fieldvoices.com/current_studies</t>
+          <t>https://www.questionspace.net/category/upcoming-studies/</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Galloway Research</t>
+          <t>Mediabarn Research</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1412,14 +1412,14 @@
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>https://www.questionspace.net/category/upcoming-studies/</t>
+          <t>https://www.mediabarnresearch.com/currentstudies/</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Mediabarn Research</t>
+          <t>Nashville Research Group</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -1429,14 +1429,14 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>https://www.mediabarnresearch.com/currentstudies/</t>
+          <t>https://www.nashvilleresearch.com/current-research-projects</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Nashville Research Group</t>
+          <t>Adler Weiner Research</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -1446,14 +1446,14 @@
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>https://www.nashvilleresearch.com/current-research-projects</t>
+          <t>https://adlerweiner.com</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Adler Weiner Research</t>
+          <t>AlphaBuzz</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -1463,14 +1463,14 @@
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>https://adlerweiner.com</t>
+          <t>https://alphabuzz.alchemer.com/</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>AlphaBuzz</t>
+          <t>AMG Research</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1480,14 +1480,14 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>https://alphabuzz.alchemer.com/</t>
+          <t>https://amgsurvey.com/</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>AMG Research</t>
+          <t>Amplify Research</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1497,14 +1497,14 @@
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>https://amgsurvey.com/</t>
+          <t>https://amplifyresearch.com/participate/</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Amplify Research</t>
+          <t>Atkins Research</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1514,14 +1514,14 @@
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>https://amplifyresearch.com/participate/</t>
+          <t>https://www.atkinsresearch.com/research-participant/respondent-signup/</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Atkins Research</t>
+          <t>Bezel Research</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1531,14 +1531,14 @@
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>https://www.atkinsresearch.com/research-participant/respondent-signup/</t>
+          <t>http://bezelrr.com/</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Bezel Research</t>
+          <t>Big Bang Recruiting</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1548,14 +1548,14 @@
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>http://bezelrr.com/</t>
+          <t>https://www.bigbangrecruiting.com/register/</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Big Bang Recruiting</t>
+          <t>Brightside Research Solutions</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -1565,14 +1565,14 @@
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>https://www.bigbangrecruiting.com/register/</t>
+          <t>https://teambrightsider.com/</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Brightside Research Solutions</t>
+          <t>Cambridge Focus</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -1582,14 +1582,14 @@
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>https://teambrightsider.com/</t>
+          <t>http://www.participatenewengland.com/</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Cambridge Focus</t>
+          <t>CEC Surveys</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -1599,14 +1599,14 @@
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>http://www.participatenewengland.com/</t>
+          <t>https://cecsurveys.com/</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>CEC Surveys</t>
+          <t>CIC Testing</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -1616,14 +1616,14 @@
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>https://cecsurveys.com/</t>
+          <t>https://www.cictesting.com/CIC/</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>CIC Testing</t>
+          <t>Citrus Labs</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -1633,14 +1633,14 @@
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>https://www.cictesting.com/CIC/</t>
+          <t>https://www.citruslabs.com/</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Citrus Labs</t>
+          <t>ClearView Research</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -1650,14 +1650,14 @@
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>https://www.citruslabs.com/</t>
+          <t>http://www.clearviewresearch.com/sign-up-now.aspx</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>ClearView Research</t>
+          <t>Collab Research</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -1667,14 +1667,14 @@
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>http://www.clearviewresearch.com/sign-up-now.aspx</t>
+          <t>https://www.collab-research.com/</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Collab Research</t>
+          <t>Compass Research</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -1684,14 +1684,14 @@
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>https://www.collab-research.com/</t>
+          <t>https://compassmarketingresearch.com/sign-up/</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Compass Research</t>
+          <t>Confide Research</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -1701,14 +1701,14 @@
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>https://compassmarketingresearch.com/sign-up/</t>
+          <t>https://confideresearch.com/Participants/signup</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Confide Research</t>
+          <t>Consumer Viewpoint</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -1718,14 +1718,14 @@
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>https://confideresearch.com/Participants/signup</t>
+          <t>https://www.paidforyouropinions.com</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Consumer Viewpoint</t>
+          <t>Contact Design</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -1735,14 +1735,14 @@
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>https://www.paidforyouropinions.com</t>
+          <t>https://yourcontacthub.com/</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Contact Design</t>
+          <t>Contract Testing</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -1752,14 +1752,14 @@
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>https://yourcontacthub.com/</t>
+          <t>https://connect.contracttesting.com/ctimvc/Account/Register</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Contract Testing</t>
+          <t>Cypher Research</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -1769,14 +1769,14 @@
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>https://connect.contracttesting.com/ctimvc/Account/Register</t>
+          <t>https://cypherresearch.com/intranet/respondent_sign_up.php</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Cypher Research</t>
+          <t>Decision Point Research</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -1786,14 +1786,14 @@
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>https://cypherresearch.com/intranet/respondent_sign_up.php</t>
+          <t>https://www.decisionpointresearch.ca</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Decision Point Research</t>
+          <t>Design Science</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -1803,14 +1803,14 @@
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>https://www.decisionpointresearch.ca</t>
+          <t>https://dscience.com/signup</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Design Science</t>
+          <t>Drive Research</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -1820,14 +1820,14 @@
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>https://dscience.com/signup</t>
+          <t>https://www.driveresearch.com/participate/</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Drive Research</t>
+          <t>Elliott Benson</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -1837,14 +1837,14 @@
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>https://www.driveresearch.com/participate/</t>
+          <t>https://www.elliottbenson.com/participate/</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Elliott Benson</t>
+          <t>EmCee Research</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -1854,14 +1854,14 @@
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>https://www.elliottbenson.com/participate/</t>
+          <t>https://emceeresearch.com/</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>EmCee Research</t>
+          <t>Engage In Depth</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -1871,14 +1871,14 @@
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>https://emceeresearch.com/</t>
+          <t>https://engageindepth.com/participate/</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Engage In Depth</t>
+          <t>Ethical Mind</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -1888,14 +1888,14 @@
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>https://engageindepth.com/participate/</t>
+          <t>https://ethicalmind.org/</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Ethical Mind</t>
+          <t>Fieldwork</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -1905,14 +1905,14 @@
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>https://ethicalmind.org/</t>
+          <t>https://www.fieldwork.com</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Fieldwork</t>
+          <t>First Court Jurors</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -1922,14 +1922,14 @@
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>https://www.fieldwork.com</t>
+          <t>https://www.firstcourt.com/jury-recruiting</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>First Court Jurors</t>
+          <t>Fleischman Field Research</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -1939,14 +1939,14 @@
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>https://www.firstcourt.com/jury-recruiting</t>
+          <t>http://www.ffrsf.com/</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Fleischman Field Research</t>
+          <t>Focus &amp; Testing</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -1956,14 +1956,14 @@
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>http://www.ffrsf.com/</t>
+          <t>https://research.focusandtesting.com/</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Focus &amp; Testing</t>
+          <t>focus 99</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -1973,14 +1973,14 @@
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>https://research.focusandtesting.com/</t>
+          <t>https://www.focus99.com/sub/</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>focus 99</t>
+          <t>Focus Corner</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -1990,14 +1990,14 @@
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>https://www.focus99.com/sub/</t>
+          <t>https://focuscorner.net/</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Focus Corner</t>
+          <t>Focus Crossroads</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -2007,14 +2007,14 @@
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>https://focuscorner.net/</t>
+          <t>https://focuscrossroads.org/research-network/join-consumer/</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Focus Crossroads</t>
+          <t>Focus Group Connection</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -2024,14 +2024,14 @@
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>https://focuscrossroads.org/research-network/join-consumer/</t>
+          <t>https://www.focusgroupconnection.com/participate/</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Focus Group Connection</t>
+          <t>Focus Group Finder</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2041,14 +2041,14 @@
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>https://www.focusgroupconnection.com/participate/</t>
+          <t>https://focusgroups.org/</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Focus Group Finder</t>
+          <t>Focus Pulse</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2058,14 +2058,14 @@
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>https://focusgroups.org/</t>
+          <t>https://focuspulseresearch.co.uk/</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Focus Pulse</t>
+          <t>Focuscope</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -2075,14 +2075,14 @@
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>https://focuspulseresearch.co.uk/</t>
+          <t>https://www.focuscope.com/join-our-community/</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Focuscope</t>
+          <t>Georgetown University (GRVP)</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2092,14 +2092,14 @@
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>https://www.focuscope.com/join-our-community/</t>
+          <t>https://grvp.georgetown.edu/</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Georgetown University (GRVP)</t>
+          <t>Griot Recruit</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2109,14 +2109,14 @@
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>https://grvp.georgetown.edu/</t>
+          <t>https://www.griotrecruit.co/</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Griot Recruit</t>
+          <t>Hagen Sinclair Research Recruiting</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -2126,14 +2126,14 @@
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>https://www.griotrecruit.co/</t>
+          <t>https://hagensinclair.com/paid-research-studies-2/</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Hagen Sinclair Research Recruiting</t>
+          <t>Horizon Group</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -2143,14 +2143,14 @@
       </c>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>https://hagensinclair.com/paid-research-studies-2/</t>
+          <t>https://www.horizongroupiowa.com/join-our-panel/</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Horizon Group</t>
+          <t>Insight Recruit</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -2160,14 +2160,14 @@
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>https://www.horizongroupiowa.com/join-our-panel/</t>
+          <t>https://insightrecruit.com/join-our-panel/</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Insight Recruit</t>
+          <t>Intact Qualitative Research</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -2177,14 +2177,14 @@
       </c>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>https://insightrecruit.com/join-our-panel/</t>
+          <t>https://www.iqrsf.com/participant-intake-form</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Intact Qualitative Research</t>
+          <t>JC Research Partners</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -2194,14 +2194,14 @@
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>https://www.iqrsf.com/participant-intake-form</t>
+          <t>https://jcresearchpartners.com/</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>JC Research Partners</t>
+          <t>Limelight by Shugoll</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -2211,14 +2211,14 @@
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>https://jcresearchpartners.com/</t>
+          <t>https://limelightbyshugoll.com/get-paid-for-your-opinion/</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Limelight by Shugoll</t>
+          <t>Local Focus Group</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -2228,14 +2228,14 @@
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>https://limelightbyshugoll.com/get-paid-for-your-opinion/</t>
+          <t>https://www.localfocusgroup.com/</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Local Focus Group</t>
+          <t>Mars Research</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -2245,14 +2245,14 @@
       </c>
       <c r="C107" s="2" t="inlineStr">
         <is>
-          <t>https://www.localfocusgroup.com/</t>
+          <t>https://joinmarsresearch.com/</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Mars Research</t>
+          <t>McCormick Group</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -2262,14 +2262,14 @@
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>https://joinmarsresearch.com/</t>
+          <t>http://mccormick-group.com/market-research.html</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>McCormick Group</t>
+          <t>MForce Research</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -2279,14 +2279,14 @@
       </c>
       <c r="C109" s="2" t="inlineStr">
         <is>
-          <t>http://mccormick-group.com/market-research.html</t>
+          <t>http://www.mforceresearch.com/</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>MForce Research</t>
+          <t>Moore Opinions</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -2296,14 +2296,14 @@
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>http://www.mforceresearch.com/</t>
+          <t>http://mooreopinions.com/</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Moore Opinions</t>
+          <t>Moore Research Services</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -2313,14 +2313,14 @@
       </c>
       <c r="C111" s="2" t="inlineStr">
         <is>
-          <t>http://mooreopinions.com/</t>
+          <t>https://www.moore-research.com/join-a-panel/</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Moore Research Services</t>
+          <t>MVG Recruiting</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -2330,14 +2330,14 @@
       </c>
       <c r="C112" s="2" t="inlineStr">
         <is>
-          <t>https://www.moore-research.com/join-a-panel/</t>
+          <t>https://mvgrecruiting.com/sign-up</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>MVG Recruiting</t>
+          <t>N.C. Litigation &amp; Jury Research Group</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -2347,14 +2347,14 @@
       </c>
       <c r="C113" s="2" t="inlineStr">
         <is>
-          <t>https://mvgrecruiting.com/sign-up</t>
+          <t>https://ncfocusgroups.com/</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>N.C. Litigation &amp; Jury Research Group</t>
+          <t>Nelson Recruiting</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -2364,14 +2364,14 @@
       </c>
       <c r="C114" s="2" t="inlineStr">
         <is>
-          <t>https://ncfocusgroups.com/</t>
+          <t>https://nelsonrecruiting.com</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Nelson Recruiting</t>
+          <t>New England Focus Group</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -2381,14 +2381,14 @@
       </c>
       <c r="C115" s="2" t="inlineStr">
         <is>
-          <t>https://nelsonrecruiting.com</t>
+          <t>https://www.newenglandfocusgroup.com/register.html</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>New England Focus Group</t>
+          <t>Newton Marketing Network</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -2398,14 +2398,14 @@
       </c>
       <c r="C116" s="2" t="inlineStr">
         <is>
-          <t>https://www.newenglandfocusgroup.com/register.html</t>
+          <t>https://newtonmarketingnetwork.com/participants/</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Newton Marketing Network</t>
+          <t>Nichols Research</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -2415,14 +2415,14 @@
       </c>
       <c r="C117" s="2" t="inlineStr">
         <is>
-          <t>https://newtonmarketingnetwork.com/participants/</t>
+          <t>https://nicholsresearch.com/registration-form/</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Nichols Research</t>
+          <t>NYC Focal (The Diamond Lists)</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -2432,14 +2432,14 @@
       </c>
       <c r="C118" s="2" t="inlineStr">
         <is>
-          <t>https://nicholsresearch.com/registration-form/</t>
+          <t>https://thediamondlists.com/join-the-list/</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>NYC Focal (The Diamond Lists)</t>
+          <t>Online Verdict</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -2449,14 +2449,14 @@
       </c>
       <c r="C119" s="2" t="inlineStr">
         <is>
-          <t>https://thediamondlists.com/join-the-list/</t>
+          <t>https://www.onlineverdict.com/jurors/signup/</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>Online Verdict</t>
+          <t>Opinions Link</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -2466,14 +2466,14 @@
       </c>
       <c r="C120" s="2" t="inlineStr">
         <is>
-          <t>https://www.onlineverdict.com/jurors/signup/</t>
+          <t>https://www.opinionslink.com</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Opinions Link</t>
+          <t>Opinions LTD</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -2483,14 +2483,14 @@
       </c>
       <c r="C121" s="2" t="inlineStr">
         <is>
-          <t>https://www.opinionslink.com</t>
+          <t>https://www.opinionsltd.com/participate/</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>Opinions LTD</t>
+          <t>Portable Insights</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -2500,14 +2500,14 @@
       </c>
       <c r="C122" s="2" t="inlineStr">
         <is>
-          <t>https://www.opinionsltd.com/participate/</t>
+          <t>https://portableinsights.com/join-our-panel</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Portable Insights</t>
+          <t>Precision Research</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -2517,14 +2517,14 @@
       </c>
       <c r="C123" s="2" t="inlineStr">
         <is>
-          <t>https://portableinsights.com/join-our-panel</t>
+          <t>https://www.opinionwizard.com/</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>Precision Research</t>
+          <t>Product Tube</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -2534,14 +2534,14 @@
       </c>
       <c r="C124" s="2" t="inlineStr">
         <is>
-          <t>https://www.opinionwizard.com/</t>
+          <t>https://web.producttube.com/signup</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>Product Tube</t>
+          <t>PVR Research</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -2551,14 +2551,14 @@
       </c>
       <c r="C125" s="2" t="inlineStr">
         <is>
-          <t>https://web.producttube.com/signup</t>
+          <t>http://www.pvr-research.com/</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>PVR Research</t>
+          <t>Q-Insights</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -2568,14 +2568,14 @@
       </c>
       <c r="C126" s="2" t="inlineStr">
         <is>
-          <t>http://www.pvr-research.com/</t>
+          <t>https://q-insights.com/</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>Q-Insights</t>
+          <t>Qual Recruit</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -2585,14 +2585,14 @@
       </c>
       <c r="C127" s="2" t="inlineStr">
         <is>
-          <t>https://q-insights.com/</t>
+          <t>https://www.qualrecruit.com/become-a-participant</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>Qual Recruit</t>
+          <t>Reckner</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -2602,14 +2602,14 @@
       </c>
       <c r="C128" s="2" t="inlineStr">
         <is>
-          <t>https://www.qualrecruit.com/become-a-participant</t>
+          <t>https://www.reckner.com</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>Reckner</t>
+          <t>Recruit and Field</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -2619,14 +2619,14 @@
       </c>
       <c r="C129" s="2" t="inlineStr">
         <is>
-          <t>https://www.reckner.com</t>
+          <t>https://www.recruitandfield.com/register-as-a-participant</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>Recruit and Field</t>
+          <t>Research Outloud</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -2636,14 +2636,14 @@
       </c>
       <c r="C130" s="2" t="inlineStr">
         <is>
-          <t>https://www.recruitandfield.com/register-as-a-participant</t>
+          <t>https://researchoutloud.com/</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>Research Outloud</t>
+          <t>Ridgeline Recruiting</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -2653,14 +2653,14 @@
       </c>
       <c r="C131" s="2" t="inlineStr">
         <is>
-          <t>https://researchoutloud.com/</t>
+          <t>https://ridgelinerecruiting.com/</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>Ridgeline Recruiting</t>
+          <t>Round2Research</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -2670,14 +2670,14 @@
       </c>
       <c r="C132" s="2" t="inlineStr">
         <is>
-          <t>https://ridgelinerecruiting.com/</t>
+          <t>https://round2research.com/</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>Round2Research</t>
+          <t>RRU Research</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -2687,14 +2687,14 @@
       </c>
       <c r="C133" s="2" t="inlineStr">
         <is>
-          <t>https://round2research.com/</t>
+          <t>https://focuspocussoftware.net/WP_RRU/Register</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>RRU Research</t>
+          <t>SIS Research</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -2704,14 +2704,14 @@
       </c>
       <c r="C134" s="2" t="inlineStr">
         <is>
-          <t>https://focuspocussoftware.net/WP_RRU/Register</t>
+          <t>https://participate.sisinternational.com/Portal/Default</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>SIS Research</t>
+          <t>Spotlight Research</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -2721,14 +2721,14 @@
       </c>
       <c r="C135" s="2" t="inlineStr">
         <is>
-          <t>https://participate.sisinternational.com/Portal/Default</t>
+          <t>https://spotlightmarketresearch.com/join-our-audience/</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>Spotlight Research</t>
+          <t>Talking Heads</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -2738,14 +2738,14 @@
       </c>
       <c r="C136" s="2" t="inlineStr">
         <is>
-          <t>https://spotlightmarketresearch.com/join-our-audience/</t>
+          <t>http://register.talkingheadsstudio.com/</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>Talking Heads</t>
+          <t>Thurs Recruiting</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -2755,14 +2755,14 @@
       </c>
       <c r="C137" s="2" t="inlineStr">
         <is>
-          <t>http://register.talkingheadsstudio.com/</t>
+          <t>https://thursrecruiting.com/</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>Thurs Recruiting</t>
+          <t>Ubinsights</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -2772,14 +2772,14 @@
       </c>
       <c r="C138" s="2" t="inlineStr">
         <is>
-          <t>https://thursrecruiting.com/</t>
+          <t>https://ubinsights.com/</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>Ubinsights</t>
+          <t>Uncover Research</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
@@ -2789,14 +2789,14 @@
       </c>
       <c r="C139" s="2" t="inlineStr">
         <is>
-          <t>https://ubinsights.com/</t>
+          <t>https://www.uncoverresearch.com/participate</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>Uncover Research</t>
+          <t>User Insight</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
@@ -2806,14 +2806,14 @@
       </c>
       <c r="C140" s="2" t="inlineStr">
         <is>
-          <t>https://www.uncoverresearch.com/participate</t>
+          <t>https://www.shareyourinsights.com/</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>User Insight</t>
+          <t>VGM (playtests)</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
@@ -2823,14 +2823,14 @@
       </c>
       <c r="C141" s="2" t="inlineStr">
         <is>
-          <t>https://www.shareyourinsights.com/</t>
+          <t>https://vgm.co/</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>VGM (playtests)</t>
+          <t>Videochat Network</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -2840,14 +2840,14 @@
       </c>
       <c r="C142" s="2" t="inlineStr">
         <is>
-          <t>https://vgm.co/</t>
+          <t>https://www.videochatnetwork.net/sign-up/</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>Videochat Network</t>
+          <t>View-Finders</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -2857,14 +2857,14 @@
       </c>
       <c r="C143" s="2" t="inlineStr">
         <is>
-          <t>https://www.videochatnetwork.net/sign-up/</t>
+          <t>https://www.view-finders.net/participant-registration-2/</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>View-Finders</t>
+          <t>WAC Research</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -2874,14 +2874,14 @@
       </c>
       <c r="C144" s="2" t="inlineStr">
         <is>
-          <t>https://www.view-finders.net/participant-registration-2/</t>
+          <t>https://wacresearch.com/data.html</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>WAC Research</t>
+          <t>Watch Me Think</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -2891,14 +2891,14 @@
       </c>
       <c r="C145" s="2" t="inlineStr">
         <is>
-          <t>https://wacresearch.com/data.html</t>
+          <t>https://watchmethink.com/contribute</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>Watch Me Think</t>
+          <t>Watchlab</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -2908,14 +2908,14 @@
       </c>
       <c r="C146" s="2" t="inlineStr">
         <is>
-          <t>https://watchmethink.com/contribute</t>
+          <t>https://watchlab.com/sign-up/</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>Watchlab</t>
+          <t>Wilkins Research Services</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -2925,14 +2925,14 @@
       </c>
       <c r="C147" s="2" t="inlineStr">
         <is>
-          <t>https://watchlab.com/sign-up/</t>
+          <t>https://wilkinsresearch.net/join-our-panel/</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>Wilkins Research Services</t>
+          <t>Winn Winn Research</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -2942,31 +2942,31 @@
       </c>
       <c r="C148" s="2" t="inlineStr">
         <is>
-          <t>https://wilkinsresearch.net/join-our-panel/</t>
+          <t>https://winnwinn.com/new/public/register</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>Winn Winn Research</t>
+          <t>20/20 Panel</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>Email-only</t>
+          <t>Unclear</t>
         </is>
       </c>
       <c r="C149" s="2" t="inlineStr">
         <is>
-          <t>https://winnwinn.com/new/public/register</t>
+          <t>https://join.2020panel.com/</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>20/20 Panel</t>
+          <t>Act One Research</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
@@ -2976,14 +2976,14 @@
       </c>
       <c r="C150" s="2" t="inlineStr">
         <is>
-          <t>https://join.2020panel.com/</t>
+          <t>https://www.actone-research.com</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>Act One Research</t>
+          <t>Advanced Focus</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
@@ -2993,14 +2993,14 @@
       </c>
       <c r="C151" s="2" t="inlineStr">
         <is>
-          <t>https://www.actone-research.com</t>
+          <t>https://ow.advancedfocus.com</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>Advanced Focus</t>
+          <t>Advanced Opinions</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -3010,14 +3010,14 @@
       </c>
       <c r="C152" s="2" t="inlineStr">
         <is>
-          <t>https://ow.advancedfocus.com</t>
+          <t>http://register.advancedopinions.com</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>Advanced Opinions</t>
+          <t>Askable</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -3027,14 +3027,14 @@
       </c>
       <c r="C153" s="2" t="inlineStr">
         <is>
-          <t>http://register.advancedopinions.com</t>
+          <t>https://www.askable.com/earn/participants</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>Askable</t>
+          <t>Blink UX</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
@@ -3044,14 +3044,14 @@
       </c>
       <c r="C154" s="2" t="inlineStr">
         <is>
-          <t>https://www.askable.com/earn/participants</t>
+          <t>https://participate.blinkux.com/</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>Blink UX</t>
+          <t>End to End Research</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
@@ -3061,14 +3061,14 @@
       </c>
       <c r="C155" s="2" t="inlineStr">
         <is>
-          <t>https://participate.blinkux.com/</t>
+          <t>https://www.endtoenduserresearch.com/participate.html</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>End to End Research</t>
+          <t>Focus Insite</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
@@ -3078,14 +3078,14 @@
       </c>
       <c r="C156" s="2" t="inlineStr">
         <is>
-          <t>https://www.endtoenduserresearch.com/participate.html</t>
+          <t>https://linktr.ee/focus_insite</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>Focus Insite</t>
+          <t>Funds for Focus</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
@@ -3095,14 +3095,14 @@
       </c>
       <c r="C157" s="2" t="inlineStr">
         <is>
-          <t>https://linktr.ee/focus_insite</t>
+          <t>https://fundsforfocus.com/</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>Funds for Focus</t>
+          <t>ISG (Information Specialists Group)</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
@@ -3112,14 +3112,14 @@
       </c>
       <c r="C158" s="2" t="inlineStr">
         <is>
-          <t>https://fundsforfocus.com/</t>
+          <t>http://www.isgpanel.com/</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>ISG (Information Specialists Group)</t>
+          <t>MacConnell Research</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -3129,14 +3129,14 @@
       </c>
       <c r="C159" s="2" t="inlineStr">
         <is>
-          <t>http://www.isgpanel.com/</t>
+          <t>http://www.macconnellresearch.com/</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>MacConnell Research</t>
+          <t>Murray Hill National</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -3146,14 +3146,14 @@
       </c>
       <c r="C160" s="2" t="inlineStr">
         <is>
-          <t>http://www.macconnellresearch.com/</t>
+          <t>https://panels.murrayhillnational.com/Portal/Default</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>Murray Hill National</t>
+          <t>NDR (National Data Research)</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -3163,14 +3163,14 @@
       </c>
       <c r="C161" s="2" t="inlineStr">
         <is>
-          <t>https://panels.murrayhillnational.com/Portal/Default</t>
+          <t>http://www.national-data.net/</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>NDR (National Data Research)</t>
+          <t>Olympic National Research</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
@@ -3180,14 +3180,14 @@
       </c>
       <c r="C162" s="2" t="inlineStr">
         <is>
-          <t>http://www.national-data.net/</t>
+          <t>https://olympicnationalprojects.com/</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>Olympic National Research</t>
+          <t>Opinions for Cash</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
@@ -3197,14 +3197,14 @@
       </c>
       <c r="C163" s="2" t="inlineStr">
         <is>
-          <t>https://olympicnationalprojects.com/</t>
+          <t>https://opinionsforcash.com/</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>Opinions for Cash</t>
+          <t>Pragmatic Research</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
@@ -3214,14 +3214,14 @@
       </c>
       <c r="C164" s="2" t="inlineStr">
         <is>
-          <t>https://opinionsforcash.com/</t>
+          <t>http://www.pragmatic-research.com/</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>Pragmatic Research</t>
+          <t>Prepare to Persuade</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
@@ -3231,14 +3231,14 @@
       </c>
       <c r="C165" s="2" t="inlineStr">
         <is>
-          <t>http://www.pragmatic-research.com/</t>
+          <t>https://www.preparetopersuade.com</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>Prepare to Persuade</t>
+          <t>Research America</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
@@ -3248,14 +3248,14 @@
       </c>
       <c r="C166" s="2" t="inlineStr">
         <is>
-          <t>https://www.preparetopersuade.com</t>
+          <t>https://researchamericainc.net/</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>Research America</t>
+          <t>Taylor Research</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
@@ -3265,14 +3265,14 @@
       </c>
       <c r="C167" s="2" t="inlineStr">
         <is>
-          <t>https://researchamericainc.net/</t>
+          <t>https://studies.taylorresearch.com/</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>Taylor Research</t>
+          <t>TELUS Digital (research)</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
@@ -3282,14 +3282,14 @@
       </c>
       <c r="C168" s="2" t="inlineStr">
         <is>
-          <t>https://studies.taylorresearch.com/</t>
+          <t>https://www.telusinternational.com/</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>TELUS Digital (research)</t>
+          <t>Truscott Research</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
@@ -3299,14 +3299,14 @@
       </c>
       <c r="C169" s="2" t="inlineStr">
         <is>
-          <t>https://www.telusinternational.com/</t>
+          <t>https://app.truscottresearch.com/register</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>Truscott Research</t>
+          <t>When Opinions Meet</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
@@ -3316,14 +3316,14 @@
       </c>
       <c r="C170" s="2" t="inlineStr">
         <is>
-          <t>https://app.truscottresearch.com/register</t>
+          <t>https://www.whenopinionsmeet.com/</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>When Opinions Meet</t>
+          <t>Wynter</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
@@ -3332,23 +3332,6 @@
         </is>
       </c>
       <c r="C171" s="2" t="inlineStr">
-        <is>
-          <t>https://www.whenopinionsmeet.com/</t>
-        </is>
-      </c>
-    </row>
-    <row r="172">
-      <c r="A172" t="inlineStr">
-        <is>
-          <t>Wynter</t>
-        </is>
-      </c>
-      <c r="B172" t="inlineStr">
-        <is>
-          <t>Unclear</t>
-        </is>
-      </c>
-      <c r="C172" s="2" t="inlineStr">
         <is>
           <t>https://wynter.com/panel</t>
         </is>
@@ -3526,7 +3509,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C169" r:id="rId168"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C170" r:id="rId169"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C171" r:id="rId170"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C172" r:id="rId171"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>